<commit_message>
Record Gas & Supply plus-5 on batch 720 and refresh the 9/17 sheet.
10132/10133/10135 Type 4 Success; 10134 HOLD missing_receipt / Ruben on PO 58948; 0040424839 HOLD missing_po / Shawn. First-pass 10128-10131 and HOLD 0040430010 left alone. No Mail.Send.

Co-authored-by: beave89atm <beave89atm@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/runs/AP-run-2026-09-17-gas-supply.xlsx
+++ b/runs/AP-run-2026-09-17-gas-supply.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Exception counts" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'AP run'!$A$1:$Q$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'AP run'!$A$1:$Q$11</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q6"/>
+  <dimension ref="A1:Q11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -902,8 +902,365 @@
       </c>
       <c r="Q6" s="2" t="inlineStr"/>
     </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Gas and Supply North Texas, LLC</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>0040425612</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr"/>
+      <c r="E7" s="2" t="n">
+        <v>240</v>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>Success</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>Finished bill (Invoice_Type 4). Header PO set=none. Misc Type 4 Shop Supplies - G&amp;S (no PO). Invoice #=0040425612 (exact PDF). Amount=240.0 after-tax (never merchandise subtotal). Fees=none (Additional Charge Fees id 11, not PPV). PPV=none. Attach status=attached. Flag status=entered-in-ai.</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr"/>
+      <c r="I7" s="2" t="inlineStr"/>
+      <c r="J7" s="2" t="n">
+        <v>10132</v>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>API Agent - 9/17/26 Gas &amp; Supply (720)</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="M7" s="2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="N7" s="2" t="inlineStr">
+        <is>
+          <t>attached</t>
+        </is>
+      </c>
+      <c r="O7" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P7" s="2" t="inlineStr">
+        <is>
+          <t>entered-with-issues</t>
+        </is>
+      </c>
+      <c r="Q7" s="2" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Gas and Supply North Texas, LLC</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>0040424839</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>59081</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>224.94</v>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>category=missing_po; owner=Shawn McKibben. HOLD (po): PO 59081 is on the invoice but not findable on live by vendor + part/WO. Will not enter as Misc Type 4 (Willbanks 209663/209664; RMP 1470159). multi-invoice-pdf page 4–5 of 4</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>missing_po</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>Shawn McKibben</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr"/>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>API Agent - 9/17/26 Gas &amp; Supply (720)</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="M8" s="2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="N8" s="2" t="inlineStr">
+        <is>
+          <t>pdf-on-vm</t>
+        </is>
+      </c>
+      <c r="O8" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P8" s="2" t="inlineStr">
+        <is>
+          <t>entered-with-issues</t>
+        </is>
+      </c>
+      <c r="Q8" s="2" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Gas and Supply North Texas, LLC</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>0040424382</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr"/>
+      <c r="E9" s="2" t="n">
+        <v>335</v>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>Success</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>Finished bill (Invoice_Type 4). Header PO set=none. Misc Type 4 Shop Supplies - G&amp;S (no PO). Invoice #=0040424382 (exact PDF). Amount=335.0 after-tax (never merchandise subtotal). Fees=$SUR485005 1 0 FUEL SURCHARGE EA 17.50 17.50 N 17.5 (Additional Charge Fees id 11, not PPV). PPV=none. Attach status=attached. Flag status=entered-in-ai.</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr"/>
+      <c r="I9" s="2" t="inlineStr"/>
+      <c r="J9" s="2" t="n">
+        <v>10133</v>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>API Agent - 9/17/26 Gas &amp; Supply (720)</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>$SUR485005 1 0 FUEL SURCHARGE EA 17.50 17.50 N 17.5</t>
+        </is>
+      </c>
+      <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="N9" s="2" t="inlineStr">
+        <is>
+          <t>attached</t>
+        </is>
+      </c>
+      <c r="O9" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P9" s="2" t="inlineStr">
+        <is>
+          <t>entered-with-issues</t>
+        </is>
+      </c>
+      <c r="Q9" s="2" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Gas and Supply North Texas, LLC</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>0040423658</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>58948</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="n">
+        <v>173.5</v>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>category=missing_receipt; owner=Ruben Perez. HOLD (receipt): no open receipt leftover on PO 58948 for Gas and Supply invoice #0040423658. PDF merch=DEWDCW210B 1.0@173.5; selected=none. Do not first-open guess. Do not invent Success. @Ruben Perez: receiving must receive the PO so AP can Select Receipts. Parent email will be Entered with issues. Outlook Entered with issues. Flag status=entered-with-issues.</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>missing_receipt</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>Ruben Perez</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="n">
+        <v>10134</v>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>API Agent - 9/17/26 Gas &amp; Supply (720)</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="M10" s="2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="N10" s="2" t="inlineStr">
+        <is>
+          <t>attached</t>
+        </is>
+      </c>
+      <c r="O10" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P10" s="2" t="inlineStr">
+        <is>
+          <t>entered-with-issues</t>
+        </is>
+      </c>
+      <c r="Q10" s="2" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Gas and Supply North Texas, LLC</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>0040421569</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr"/>
+      <c r="E11" s="2" t="n">
+        <v>331.5</v>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>Success</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>Finished bill (Invoice_Type 4). Header PO set=none. Misc Type 4 Shop Supplies - G&amp;S (no PO). Invoice #=0040421569 (exact PDF). Amount=331.5 after-tax (never merchandise subtotal). Fees=$SUR485005 1 0 FUEL SURCHARGE EA 17.50 17.50 N 17.5 (Additional Charge Fees id 11, not PPV). PPV=none. Attach status=attached. Flag status=entered-in-ai.</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr"/>
+      <c r="I11" s="2" t="inlineStr"/>
+      <c r="J11" s="2" t="n">
+        <v>10135</v>
+      </c>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>API Agent - 9/17/26 Gas &amp; Supply (720)</t>
+        </is>
+      </c>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>$SUR485005 1 0 FUEL SURCHARGE EA 17.50 17.50 N 17.5</t>
+        </is>
+      </c>
+      <c r="M11" s="2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="N11" s="2" t="inlineStr">
+        <is>
+          <t>attached</t>
+        </is>
+      </c>
+      <c r="O11" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P11" s="2" t="inlineStr">
+        <is>
+          <t>entered-in-ai</t>
+        </is>
+      </c>
+      <c r="Q11" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:Q6"/>
+  <autoFilter ref="A1:Q11"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -914,7 +1271,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:B3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -940,6 +1297,16 @@
         </is>
       </c>
       <c r="B2" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>missing_receipt</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Record Gas & Supply plus-10 on batch 720 and refresh the 9/17 sheet.
9/18 A3050 pack: 10136 Success 0040438494; four HOLD missing_po / Shawn on PO 59081. Prior Success 10128-10135 and HOLDs left alone. No Mail.Send.

Co-authored-by: beave89atm <beave89atm@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/runs/AP-run-2026-09-17-gas-supply.xlsx
+++ b/runs/AP-run-2026-09-17-gas-supply.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Exception counts" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'AP run'!$A$1:$Q$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'AP run'!$A$1:$Q$16</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q11"/>
+  <dimension ref="A1:Q16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -789,7 +789,7 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>category=missing_po; owner=Misty McCoy / Transfer AP. HOLD (po): PO 59081 is on the invoice but not findable on live by vendor + part/WO. Will not enter as Misc Type 4 (Willbanks 209663/209664; RMP 1470159).</t>
+          <t>category=missing_po; owner=Shawn McKibben. HOLD (po): PO 59081 is on the invoice but not findable on live by vendor + part/WO. Will not enter as Misc Type 4 (Willbanks 209663/209664; RMP 1470159).</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
@@ -799,7 +799,7 @@
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>Misty McCoy / Transfer AP</t>
+          <t>Shawn McKibben</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr"/>
@@ -1259,8 +1259,383 @@
       </c>
       <c r="Q11" s="2" t="inlineStr"/>
     </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Gas and Supply North Texas, LLC</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>0040438494</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr"/>
+      <c r="E12" s="2" t="n">
+        <v>331.5</v>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>Success</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>Finished bill (Invoice_Type 4). Header PO set=none. Misc Type 4 Shop Supplies - G&amp;S (no PO). Invoice #=0040438494 (exact PDF). Amount=331.5 after-tax (never merchandise subtotal). Fees=$SUR485005 1 0 FUEL SURCHARGE EA 17.50 17.50 N 17.5 (Additional Charge Fees id 11, not PPV). PPV=none. Attach status=attached. Flag status=entered-in-ai.</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr"/>
+      <c r="I12" s="2" t="inlineStr"/>
+      <c r="J12" s="2" t="n">
+        <v>10136</v>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>API Agent - 9/17/26 Gas &amp; Supply (720)</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>$SUR485005 1 0 FUEL SURCHARGE EA 17.50 17.50 N 17.5</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="N12" s="2" t="inlineStr">
+        <is>
+          <t>attached</t>
+        </is>
+      </c>
+      <c r="O12" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P12" s="2" t="inlineStr">
+        <is>
+          <t>entered-with-issues</t>
+        </is>
+      </c>
+      <c r="Q12" s="2" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Gas and Supply North Texas, LLC</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>0040438057</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>59081</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="n">
+        <v>36.12</v>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>category=missing_po; owner=Shawn McKibben. HOLD (po): PO 59081 is on the invoice but not findable on live by vendor + part/WO. Will not enter as Misc Type 4 (Willbanks 209663/209664; RMP 1470159). multi-invoice-pdf page 1–2 of 7</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>missing_po</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>Shawn McKibben</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr"/>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>API Agent - 9/17/26 Gas &amp; Supply (720)</t>
+        </is>
+      </c>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="M13" s="2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="N13" s="2" t="inlineStr">
+        <is>
+          <t>pdf-on-vm</t>
+        </is>
+      </c>
+      <c r="O13" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P13" s="2" t="inlineStr">
+        <is>
+          <t>entered-with-issues</t>
+        </is>
+      </c>
+      <c r="Q13" s="2" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Gas and Supply North Texas, LLC</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>0040438056</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>59081</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="n">
+        <v>207.53</v>
+      </c>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>category=missing_po; owner=Shawn McKibben. HOLD (po): PO 59081 is on the invoice but not findable on live by vendor + part/WO. Will not enter as Misc Type 4 (Willbanks 209663/209664; RMP 1470159). multi-invoice-pdf page 7–8 of 7</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>missing_po</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>Shawn McKibben</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr"/>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>API Agent - 9/17/26 Gas &amp; Supply (720)</t>
+        </is>
+      </c>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="N14" s="2" t="inlineStr">
+        <is>
+          <t>pdf-on-vm</t>
+        </is>
+      </c>
+      <c r="O14" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P14" s="2" t="inlineStr">
+        <is>
+          <t>entered-with-issues</t>
+        </is>
+      </c>
+      <c r="Q14" s="2" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Gas and Supply North Texas, LLC</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>0040438055</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>59081</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="n">
+        <v>27.82</v>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>category=missing_po; owner=Shawn McKibben. HOLD (po): PO 59081 is on the invoice but not findable on live by vendor + part/WO. Will not enter as Misc Type 4 (Willbanks 209663/209664; RMP 1470159). multi-invoice-pdf page 8–8 of 7</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>missing_po</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>Shawn McKibben</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr"/>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>API Agent - 9/17/26 Gas &amp; Supply (720)</t>
+        </is>
+      </c>
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="M15" s="2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="N15" s="2" t="inlineStr">
+        <is>
+          <t>pdf-on-vm</t>
+        </is>
+      </c>
+      <c r="O15" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P15" s="2" t="inlineStr">
+        <is>
+          <t>entered-with-issues</t>
+        </is>
+      </c>
+      <c r="Q15" s="2" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Gas and Supply North Texas, LLC</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>0040438053</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>59081</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="n">
+        <v>182.5</v>
+      </c>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>category=missing_po; owner=Shawn McKibben. HOLD (po): PO 59081 is on the invoice but not findable on live by vendor + part/WO. Will not enter as Misc Type 4 (Willbanks 209663/209664; RMP 1470159). multi-invoice-pdf page 6–7 of 7</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>missing_po</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>Shawn McKibben</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr"/>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>API Agent - 9/17/26 Gas &amp; Supply (720)</t>
+        </is>
+      </c>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="M16" s="2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="N16" s="2" t="inlineStr">
+        <is>
+          <t>pdf-on-vm</t>
+        </is>
+      </c>
+      <c r="O16" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P16" s="2" t="inlineStr">
+        <is>
+          <t>entered-with-issues</t>
+        </is>
+      </c>
+      <c r="Q16" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:Q11"/>
+  <autoFilter ref="A1:Q16"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1297,7 +1672,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3">

</xml_diff>

<commit_message>
Add Lines-K on remaining Gas batch 720 Successes and refresh the sheet.
Live PUT on 10128–10133 and 10136 using Shop Supplies - G&S id 31. Leave
10135 and HOLDs untouched. Invoice_Amount now matches each PDF after-tax
total. NOTE-42 Why on Success rows.

Co-authored-by: beave89atm <beave89atm@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/runs/AP-run-2026-09-17-gas-supply.xlsx
+++ b/runs/AP-run-2026-09-17-gas-supply.xlsx
@@ -584,7 +584,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Finished bill (Invoice_Type 4). Header PO set=none. Misc Type 4 Shop Supplies - G&amp;S (no PO). Invoice #=0040435122 (exact PDF). Amount=120.0 after-tax (never merchandise subtotal). Fees=none (Additional Charge Fees id 11, not PPV). PPV=none. Attach status=attached. Flag status=entered-in-ai.</t>
+          <t>Finished bill (Invoice_Type 4). Header PO set=none. Misc Type 4 Lines-K Shop Supplies - G&amp;S (no PO). Invoice #=0040435122 (exact PDF). Amount=120.0 after-tax (never merchandise subtotal). Fees=none (Additional Charge Fees id 11, not PPV). PPV=none. Attach status=attached. Flag status=entered-in-ai.</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -651,7 +651,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Finished bill (Invoice_Type 4). Header PO set=none. Misc Type 4 Shop Supplies - G&amp;S (no PO). Invoice #=0040434973 (exact PDF). Amount=192.0 after-tax (never merchandise subtotal). Fees=none (Additional Charge Fees id 11, not PPV). PPV=none. Attach status=attached. Flag status=entered-in-ai.</t>
+          <t>Finished bill (Invoice_Type 4). Header PO set=none. Misc Type 4 Lines-K Shop Supplies - G&amp;S (no PO). Invoice #=0040434973 (exact PDF). Amount=192.0 after-tax (never merchandise subtotal). Fees=none (Additional Charge Fees id 11, not PPV). PPV=none. Attach status=attached. Flag status=entered-in-ai.</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr"/>
@@ -718,7 +718,7 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Finished bill (Invoice_Type 4). Header PO set=none. Misc Type 4 Shop Supplies - G&amp;S (no PO). Invoice #=0040431060 (exact PDF). Amount=245.5 after-tax (never merchandise subtotal). Fees=$SUR485005 1 0 FUEL SURCHARGE EA 17.50 17.50 N 17.5 (Additional Charge Fees id 11, not PPV). PPV=none. Attach status=attached. Flag status=entered-in-ai.</t>
+          <t>Finished bill (Invoice_Type 4). Header PO set=none. Misc Type 4 Lines-K Shop Supplies - G&amp;S (no PO). Invoice #=0040431060 (exact PDF). Amount=245.5 after-tax (never merchandise subtotal). Fees=$SUR485005 1 0 FUEL SURCHARGE EA 17.50 17.50 N 17.5 (Additional Charge Fees id 11, not PPV). PPV=none. Attach status=attached. Flag status=entered-in-ai.</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -862,7 +862,7 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Finished bill (Invoice_Type 4). Header PO set=none. Misc Type 4 Shop Supplies - G&amp;S (no PO). Invoice #=0040425657 (exact PDF). Amount=216.0 after-tax (never merchandise subtotal). Fees=none (Additional Charge Fees id 11, not PPV). PPV=none. Attach status=attached. Flag status=entered-in-ai.</t>
+          <t>Finished bill (Invoice_Type 4). Header PO set=none. Misc Type 4 Lines-K Shop Supplies - G&amp;S (no PO). Invoice #=0040425657 (exact PDF). Amount=216.0 after-tax (never merchandise subtotal). Fees=none (Additional Charge Fees id 11, not PPV). PPV=none. Attach status=attached. Flag status=entered-in-ai.</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -929,7 +929,7 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Finished bill (Invoice_Type 4). Header PO set=none. Misc Type 4 Shop Supplies - G&amp;S (no PO). Invoice #=0040425612 (exact PDF). Amount=240.0 after-tax (never merchandise subtotal). Fees=none (Additional Charge Fees id 11, not PPV). PPV=none. Attach status=attached. Flag status=entered-in-ai.</t>
+          <t>Finished bill (Invoice_Type 4). Header PO set=none. Misc Type 4 Lines-K Shop Supplies - G&amp;S (no PO). Invoice #=0040425612 (exact PDF). Amount=240.0 after-tax (never merchandise subtotal). Fees=none (Additional Charge Fees id 11, not PPV). PPV=none. Attach status=attached. Flag status=entered-in-ai.</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr"/>
@@ -964,7 +964,7 @@
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>entered-with-issues</t>
+          <t>entered-in-ai</t>
         </is>
       </c>
       <c r="Q7" s="2" t="inlineStr"/>
@@ -1073,7 +1073,7 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>Finished bill (Invoice_Type 4). Header PO set=none. Misc Type 4 Shop Supplies - G&amp;S (no PO). Invoice #=0040424382 (exact PDF). Amount=335.0 after-tax (never merchandise subtotal). Fees=$SUR485005 1 0 FUEL SURCHARGE EA 17.50 17.50 N 17.5 (Additional Charge Fees id 11, not PPV). PPV=none. Attach status=attached. Flag status=entered-in-ai.</t>
+          <t>Finished bill (Invoice_Type 4). Header PO set=none. Misc Type 4 Lines-K Shop Supplies - G&amp;S (no PO). Invoice #=0040424382 (exact PDF). Amount=335.0 after-tax (never merchandise subtotal). Fees=$SUR485005 1 0 FUEL SURCHARGE EA 17.50 17.50 N 17.5 (Additional Charge Fees id 11, not PPV). PPV=none. Attach status=attached. Flag status=entered-in-ai.</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr"/>
@@ -1108,7 +1108,7 @@
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>entered-with-issues</t>
+          <t>entered-in-ai</t>
         </is>
       </c>
       <c r="Q9" s="2" t="inlineStr"/>
@@ -1219,7 +1219,7 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>Finished bill (Invoice_Type 4). Header PO set=none. Misc Type 4 Shop Supplies - G&amp;S (no PO). Invoice #=0040421569 (exact PDF). Amount=331.5 after-tax (never merchandise subtotal). Fees=$SUR485005 1 0 FUEL SURCHARGE EA 17.50 17.50 N 17.5 (Additional Charge Fees id 11, not PPV). PPV=none. Attach status=attached. Flag status=entered-in-ai.</t>
+          <t>Finished bill (Invoice_Type 4). Header PO set=none. Misc Type 4 Lines-K Shop Supplies - G&amp;S (no PO). Invoice #=0040421569 (exact PDF). Amount=331.5 after-tax (never merchandise subtotal). Fees=$SUR485005 1 0 FUEL SURCHARGE EA 17.50 17.50 N 17.5 (Additional Charge Fees id 11, not PPV). PPV=none. Attach status=attached. Flag status=entered-in-ai.</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr"/>
@@ -1286,7 +1286,7 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Finished bill (Invoice_Type 4). Header PO set=none. Misc Type 4 Shop Supplies - G&amp;S (no PO). Invoice #=0040438494 (exact PDF). Amount=331.5 after-tax (never merchandise subtotal). Fees=$SUR485005 1 0 FUEL SURCHARGE EA 17.50 17.50 N 17.5 (Additional Charge Fees id 11, not PPV). PPV=none. Attach status=attached. Flag status=entered-in-ai.</t>
+          <t>Finished bill (Invoice_Type 4). Header PO set=none. Misc Type 4 Lines-K Shop Supplies - G&amp;S (no PO). Invoice #=0040438494 (exact PDF). Amount=331.5 after-tax (never merchandise subtotal). Fees=$SUR485005 1 0 FUEL SURCHARGE EA 17.50 17.50 N 17.5 (Additional Charge Fees id 11, not PPV). PPV=none. Attach status=attached. Flag status=entered-in-ai.</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
Record Gas plus-15: three PO-cited bills, no finishable no-PO left.
0040417672 / 0040414962 HOLD missing_po Shawn (no Type 4). 0040414821
10137 Type 3 over-PPV moved to Transfer AP with @Shawn; receipts not
selected. Refresh the 9/17 gas sheet.

Co-authored-by: beave89atm <beave89atm@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/runs/AP-run-2026-09-17-gas-supply.xlsx
+++ b/runs/AP-run-2026-09-17-gas-supply.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Exception counts" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'AP run'!$A$1:$Q$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'AP run'!$A$1:$Q$19</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q16"/>
+  <dimension ref="A1:Q19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1634,8 +1634,241 @@
       </c>
       <c r="Q16" s="2" t="inlineStr"/>
     </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Gas and Supply North Texas, LLC</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>0040417672</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>59081</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="n">
+        <v>3856.77</v>
+      </c>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>category=missing_po; owner=Shawn McKibben. HOLD (po): PO 59081 is on the invoice but not findable on live by vendor + part/WO. Will not enter as Misc Type 4 (Willbanks 209663/209664; RMP 1470159).</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>missing_po</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>Shawn McKibben</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr"/>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>API Agent - 9/17/26 Gas &amp; Supply (720)</t>
+        </is>
+      </c>
+      <c r="L17" s="2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="M17" s="2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="N17" s="2" t="inlineStr">
+        <is>
+          <t>pdf-on-vm</t>
+        </is>
+      </c>
+      <c r="O17" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P17" s="2" t="inlineStr">
+        <is>
+          <t>ai-hold</t>
+        </is>
+      </c>
+      <c r="Q17" s="2" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Gas and Supply North Texas, LLC</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>0040414962</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>59006</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="n">
+        <v>7840.8</v>
+      </c>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>category=missing_po; owner=Shawn McKibben. HOLD (po): PO 59006 is on the invoice but not findable on live by vendor + part/WO. Will not enter as Misc Type 4 (Willbanks 209663/209664; RMP 1470159). multi-invoice-pdf page 2–2 of 2</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>missing_po</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>Shawn McKibben</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr"/>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>API Agent - 9/17/26 Gas &amp; Supply (720)</t>
+        </is>
+      </c>
+      <c r="L18" s="2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="M18" s="2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="N18" s="2" t="inlineStr">
+        <is>
+          <t>pdf-on-vm</t>
+        </is>
+      </c>
+      <c r="O18" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P18" s="2" t="inlineStr">
+        <is>
+          <t>entered-with-issues</t>
+        </is>
+      </c>
+      <c r="Q18" s="2" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Gas and Supply North Texas, LLC</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>0040414821</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>58948</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="n">
+        <v>293</v>
+      </c>
+      <c r="F19" s="4" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>category=price_variance; owner=Shawn McKibben. HOLD (price-does-not-match): leftover vs invoice line is over the PPV gate. Do not Select Receipts on that line. @Shawn McKibben: purchasing must unreceive, change the PO price, and re-receive. Outlook Entered with issues. Flag status=entered-with-issues. Transfer AP status=moved batch_id=375 comment='@Shawn McKibben HOLD (price-does-not-match) on Gas and Supply 0040414821 PO 58948 PDF $293.00. Leftover vs invoice line is over the PPV gate. Receipts were NOT selected so purchasing can unreceive, change the PO price, and re-receive. Do not alter receipt unit price in GI.' @mention=Comments persisted @Shawn McKibben. No mention/notify field on the record. Dedicated GET comments/mentions/notifications → [{'suffix': 'comments', 'http': 404}, {'suffix': 'mentions', 'http': 404}, {'suffix': 'notifications', 'http': 404}]. @mention notify not confirmed — cannot claim a user alert fired..</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>price_variance</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>Shawn McKibben</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="n">
+        <v>10137</v>
+      </c>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>TRANSFER AP (375)</t>
+        </is>
+      </c>
+      <c r="L19" s="2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="M19" s="2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="N19" s="2" t="inlineStr">
+        <is>
+          <t>attached</t>
+        </is>
+      </c>
+      <c r="O19" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P19" s="2" t="inlineStr">
+        <is>
+          <t>entered-with-issues</t>
+        </is>
+      </c>
+      <c r="Q19" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:Q16"/>
+  <autoFilter ref="A1:Q19"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1646,7 +1879,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1672,7 +1905,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="3">
@@ -1682,6 +1915,16 @@
         </is>
       </c>
       <c r="B3" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>price_variance</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Finish Gas 10134 and 10137 after Shawn PO 58948 leftovers.
Select Receipts 24282 1@173.50 on 0040423658 / 10134 (was missing_receipt)
and 24283 2@146.50 on 0040414821 / 10137 (was over-PPV on Transfer AP).
Posted amounts match PDF; 10137 moved back to batch 720. PO 59081/59006
still have no receipts. Sheet refreshed. No Mail.Send.

Co-authored-by: beave89atm <beave89atm@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/runs/AP-run-2026-09-17-gas-supply.xlsx
+++ b/runs/AP-run-2026-09-17-gas-supply.xlsx
@@ -1137,26 +1137,18 @@
       <c r="E10" s="2" t="n">
         <v>173.5</v>
       </c>
-      <c r="F10" s="4" t="inlineStr">
-        <is>
-          <t>HOLD</t>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>Success</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>category=missing_receipt; owner=Ruben Perez. HOLD (receipt): no open receipt leftover on PO 58948 for Gas and Supply invoice #0040423658. PDF merch=DEWDCW210B 1.0@173.5; selected=none. Do not first-open guess. Do not invent Success. @Ruben Perez: receiving must receive the PO so AP can Select Receipts. Parent email will be Entered with issues. Outlook Entered with issues. Flag status=entered-with-issues.</t>
-        </is>
-      </c>
-      <c r="H10" s="2" t="inlineStr">
-        <is>
-          <t>missing_receipt</t>
-        </is>
-      </c>
-      <c r="I10" s="2" t="inlineStr">
-        <is>
-          <t>Ruben Perez</t>
-        </is>
-      </c>
+          <t>Finished bill (Invoice_Type 3). Header PO set=58948. Select Receipts 24282 1@173.5 on PO 58948. Invoice #=0040423658 (exact PDF). Amount=173.5 after-tax (never merchandise subtotal). Fees=none (Additional Charge Fees id 11, not PPV). PPV=none. Attach status=attached. Finish Select Receipts selected ids=[24282] fees=none ppv=none. Flag status=entered-in-ai.</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr"/>
+      <c r="I10" s="2" t="inlineStr"/>
       <c r="J10" s="2" t="n">
         <v>10134</v>
       </c>
@@ -1187,7 +1179,7 @@
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>entered-with-issues</t>
+          <t>entered-in-ai</t>
         </is>
       </c>
       <c r="Q10" s="2" t="inlineStr"/>
@@ -1812,32 +1804,24 @@
       <c r="E19" s="2" t="n">
         <v>293</v>
       </c>
-      <c r="F19" s="4" t="inlineStr">
-        <is>
-          <t>HOLD</t>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>Success</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>category=price_variance; owner=Shawn McKibben. HOLD (price-does-not-match): leftover vs invoice line is over the PPV gate. Do not Select Receipts on that line. @Shawn McKibben: purchasing must unreceive, change the PO price, and re-receive. Outlook Entered with issues. Flag status=entered-with-issues. Transfer AP status=moved batch_id=375 comment='@Shawn McKibben HOLD (price-does-not-match) on Gas and Supply 0040414821 PO 58948 PDF $293.00. Leftover vs invoice line is over the PPV gate. Receipts were NOT selected so purchasing can unreceive, change the PO price, and re-receive. Do not alter receipt unit price in GI.' @mention=Comments persisted @Shawn McKibben. No mention/notify field on the record. Dedicated GET comments/mentions/notifications → [{'suffix': 'comments', 'http': 404}, {'suffix': 'mentions', 'http': 404}, {'suffix': 'notifications', 'http': 404}]. @mention notify not confirmed — cannot claim a user alert fired..</t>
-        </is>
-      </c>
-      <c r="H19" s="2" t="inlineStr">
-        <is>
-          <t>price_variance</t>
-        </is>
-      </c>
-      <c r="I19" s="2" t="inlineStr">
-        <is>
-          <t>Shawn McKibben</t>
-        </is>
-      </c>
+          <t>Finished bill (Invoice_Type 3). Header PO set=58948. Select Receipts 24283 2@146.5 on PO 58948. Invoice #=0040414821 (exact PDF). Amount=293.0 after-tax (never merchandise subtotal). Fees=none (Additional Charge Fees id 11, not PPV). PPV=none. Attach status=attached. Finish Select Receipts selected ids=[24283] fees=none ppv=none. Flag status=entered-in-ai.</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr"/>
+      <c r="I19" s="2" t="inlineStr"/>
       <c r="J19" s="2" t="n">
         <v>10137</v>
       </c>
       <c r="K19" s="2" t="inlineStr">
         <is>
-          <t>TRANSFER AP (375)</t>
+          <t>API Agent - 9/17/26 Gas &amp; Supply (720)</t>
         </is>
       </c>
       <c r="L19" s="2" t="inlineStr">
@@ -1862,7 +1846,7 @@
       </c>
       <c r="P19" s="2" t="inlineStr">
         <is>
-          <t>entered-with-issues</t>
+          <t>entered-in-ai</t>
         </is>
       </c>
       <c r="Q19" s="2" t="inlineStr"/>
@@ -1879,7 +1863,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:B2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1908,26 +1892,6 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>missing_receipt</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>price_variance</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>1</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Enter Gas 59081/59006 Type 3 HOLDs; PO exists, 0 received.
PO header/lines are on live purchase_lines (lookup 7083 / 7008) but
Received_Quantity is 0 and the receipts list has no leftovers. Entered
the eight cited invoices on batch 720 as Type 3 missing_receipt — not
Type 4, not Success.

Co-authored-by: beave89atm <beave89atm@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/runs/AP-run-2026-09-17-gas-supply.xlsx
+++ b/runs/AP-run-2026-09-17-gas-supply.xlsx
@@ -766,43 +766,33 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>0040430010</t>
+          <t>0040425657</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>59081</t>
-        </is>
-      </c>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr"/>
       <c r="E5" s="2" t="n">
-        <v>14</v>
-      </c>
-      <c r="F5" s="4" t="inlineStr">
-        <is>
-          <t>HOLD</t>
+        <v>216</v>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>Success</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>category=missing_po; owner=Shawn McKibben. HOLD (po): PO 59081 is on the invoice but not findable on live by vendor + part/WO. Will not enter as Misc Type 4 (Willbanks 209663/209664; RMP 1470159).</t>
-        </is>
-      </c>
-      <c r="H5" s="2" t="inlineStr">
-        <is>
-          <t>missing_po</t>
-        </is>
-      </c>
-      <c r="I5" s="2" t="inlineStr">
-        <is>
-          <t>Shawn McKibben</t>
-        </is>
-      </c>
-      <c r="J5" s="2" t="inlineStr"/>
+          <t>Finished bill (Invoice_Type 4). Header PO set=none. Misc Type 4 Lines-K Shop Supplies - G&amp;S (no PO). Invoice #=0040425657 (exact PDF). Amount=216.0 after-tax (never merchandise subtotal). Fees=none (Additional Charge Fees id 11, not PPV). PPV=none. Attach status=attached. Flag status=entered-in-ai.</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr"/>
+      <c r="I5" s="2" t="inlineStr"/>
+      <c r="J5" s="2" t="n">
+        <v>10131</v>
+      </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
           <t>API Agent - 9/17/26 Gas &amp; Supply (720)</t>
@@ -820,7 +810,7 @@
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>pdf-on-vm</t>
+          <t>attached</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
@@ -830,7 +820,7 @@
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>ai-hold</t>
+          <t>entered-in-ai</t>
         </is>
       </c>
       <c r="Q5" s="2" t="inlineStr"/>
@@ -843,7 +833,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>0040425657</t>
+          <t>0040425612</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -853,7 +843,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr"/>
       <c r="E6" s="2" t="n">
-        <v>216</v>
+        <v>240</v>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
@@ -862,13 +852,13 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Finished bill (Invoice_Type 4). Header PO set=none. Misc Type 4 Lines-K Shop Supplies - G&amp;S (no PO). Invoice #=0040425657 (exact PDF). Amount=216.0 after-tax (never merchandise subtotal). Fees=none (Additional Charge Fees id 11, not PPV). PPV=none. Attach status=attached. Flag status=entered-in-ai.</t>
+          <t>Finished bill (Invoice_Type 4). Header PO set=none. Misc Type 4 Lines-K Shop Supplies - G&amp;S (no PO). Invoice #=0040425612 (exact PDF). Amount=240.0 after-tax (never merchandise subtotal). Fees=none (Additional Charge Fees id 11, not PPV). PPV=none. Attach status=attached. Flag status=entered-in-ai.</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
       <c r="I6" s="2" t="inlineStr"/>
       <c r="J6" s="2" t="n">
-        <v>10131</v>
+        <v>10132</v>
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
@@ -910,7 +900,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>0040425612</t>
+          <t>0040424382</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -920,7 +910,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr"/>
       <c r="E7" s="2" t="n">
-        <v>240</v>
+        <v>335</v>
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
@@ -929,13 +919,13 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Finished bill (Invoice_Type 4). Header PO set=none. Misc Type 4 Lines-K Shop Supplies - G&amp;S (no PO). Invoice #=0040425612 (exact PDF). Amount=240.0 after-tax (never merchandise subtotal). Fees=none (Additional Charge Fees id 11, not PPV). PPV=none. Attach status=attached. Flag status=entered-in-ai.</t>
+          <t>Finished bill (Invoice_Type 4). Header PO set=none. Misc Type 4 Lines-K Shop Supplies - G&amp;S (no PO). Invoice #=0040424382 (exact PDF). Amount=335.0 after-tax (never merchandise subtotal). Fees=$SUR485005 1 0 FUEL SURCHARGE EA 17.50 17.50 N 17.5 (Additional Charge Fees id 11, not PPV). PPV=none. Attach status=attached. Flag status=entered-in-ai.</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr"/>
       <c r="I7" s="2" t="inlineStr"/>
       <c r="J7" s="2" t="n">
-        <v>10132</v>
+        <v>10133</v>
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
@@ -944,7 +934,7 @@
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>$SUR485005 1 0 FUEL SURCHARGE EA 17.50 17.50 N 17.5</t>
         </is>
       </c>
       <c r="M7" s="2" t="inlineStr">
@@ -977,7 +967,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>0040424839</t>
+          <t>0040423658</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -987,33 +977,27 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>59081</t>
+          <t>58948</t>
         </is>
       </c>
       <c r="E8" s="2" t="n">
-        <v>224.94</v>
-      </c>
-      <c r="F8" s="4" t="inlineStr">
-        <is>
-          <t>HOLD</t>
+        <v>173.5</v>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>Success</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>category=missing_po; owner=Shawn McKibben. HOLD (po): PO 59081 is on the invoice but not findable on live by vendor + part/WO. Will not enter as Misc Type 4 (Willbanks 209663/209664; RMP 1470159). multi-invoice-pdf page 4–5 of 4</t>
-        </is>
-      </c>
-      <c r="H8" s="2" t="inlineStr">
-        <is>
-          <t>missing_po</t>
-        </is>
-      </c>
-      <c r="I8" s="2" t="inlineStr">
-        <is>
-          <t>Shawn McKibben</t>
-        </is>
-      </c>
-      <c r="J8" s="2" t="inlineStr"/>
+          <t>Finished bill (Invoice_Type 3). Header PO set=58948. Select Receipts 24282 1@173.5 on PO 58948. Invoice #=0040423658 (exact PDF). Amount=173.5 after-tax (never merchandise subtotal). Fees=none (Additional Charge Fees id 11, not PPV). PPV=none. Attach status=attached. Finish Select Receipts selected ids=[24282] fees=none ppv=none. Flag status=entered-in-ai.</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr"/>
+      <c r="I8" s="2" t="inlineStr"/>
+      <c r="J8" s="2" t="n">
+        <v>10134</v>
+      </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
           <t>API Agent - 9/17/26 Gas &amp; Supply (720)</t>
@@ -1031,7 +1015,7 @@
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>pdf-on-vm</t>
+          <t>attached</t>
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr">
@@ -1041,7 +1025,7 @@
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>entered-with-issues</t>
+          <t>entered-in-ai</t>
         </is>
       </c>
       <c r="Q8" s="2" t="inlineStr"/>
@@ -1054,17 +1038,17 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>0040424382</t>
+          <t>0040421569</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr"/>
       <c r="E9" s="2" t="n">
-        <v>335</v>
+        <v>331.5</v>
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
@@ -1073,13 +1057,13 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>Finished bill (Invoice_Type 4). Header PO set=none. Misc Type 4 Lines-K Shop Supplies - G&amp;S (no PO). Invoice #=0040424382 (exact PDF). Amount=335.0 after-tax (never merchandise subtotal). Fees=$SUR485005 1 0 FUEL SURCHARGE EA 17.50 17.50 N 17.5 (Additional Charge Fees id 11, not PPV). PPV=none. Attach status=attached. Flag status=entered-in-ai.</t>
+          <t>Finished bill (Invoice_Type 4). Header PO set=none. Misc Type 4 Lines-K Shop Supplies - G&amp;S (no PO). Invoice #=0040421569 (exact PDF). Amount=331.5 after-tax (never merchandise subtotal). Fees=$SUR485005 1 0 FUEL SURCHARGE EA 17.50 17.50 N 17.5 (Additional Charge Fees id 11, not PPV). PPV=none. Attach status=attached. Flag status=entered-in-ai.</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr"/>
       <c r="I9" s="2" t="inlineStr"/>
       <c r="J9" s="2" t="n">
-        <v>10133</v>
+        <v>10135</v>
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
@@ -1121,21 +1105,17 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>0040423658</t>
+          <t>0040438494</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>58948</t>
-        </is>
-      </c>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr"/>
       <c r="E10" s="2" t="n">
-        <v>173.5</v>
+        <v>331.5</v>
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
@@ -1144,13 +1124,13 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Finished bill (Invoice_Type 3). Header PO set=58948. Select Receipts 24282 1@173.5 on PO 58948. Invoice #=0040423658 (exact PDF). Amount=173.5 after-tax (never merchandise subtotal). Fees=none (Additional Charge Fees id 11, not PPV). PPV=none. Attach status=attached. Finish Select Receipts selected ids=[24282] fees=none ppv=none. Flag status=entered-in-ai.</t>
+          <t>Finished bill (Invoice_Type 4). Header PO set=none. Misc Type 4 Lines-K Shop Supplies - G&amp;S (no PO). Invoice #=0040438494 (exact PDF). Amount=331.5 after-tax (never merchandise subtotal). Fees=$SUR485005 1 0 FUEL SURCHARGE EA 17.50 17.50 N 17.5 (Additional Charge Fees id 11, not PPV). PPV=none. Attach status=attached. Flag status=entered-in-ai.</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr"/>
       <c r="I10" s="2" t="inlineStr"/>
       <c r="J10" s="2" t="n">
-        <v>10134</v>
+        <v>10136</v>
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
@@ -1159,7 +1139,7 @@
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>$SUR485005 1 0 FUEL SURCHARGE EA 17.50 17.50 N 17.5</t>
         </is>
       </c>
       <c r="M10" s="2" t="inlineStr">
@@ -1179,7 +1159,7 @@
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>entered-in-ai</t>
+          <t>entered-with-issues</t>
         </is>
       </c>
       <c r="Q10" s="2" t="inlineStr"/>
@@ -1192,17 +1172,21 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>0040421569</t>
+          <t>0040414821</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr"/>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>58948</t>
+        </is>
+      </c>
       <c r="E11" s="2" t="n">
-        <v>331.5</v>
+        <v>293</v>
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
@@ -1211,13 +1195,13 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>Finished bill (Invoice_Type 4). Header PO set=none. Misc Type 4 Lines-K Shop Supplies - G&amp;S (no PO). Invoice #=0040421569 (exact PDF). Amount=331.5 after-tax (never merchandise subtotal). Fees=$SUR485005 1 0 FUEL SURCHARGE EA 17.50 17.50 N 17.5 (Additional Charge Fees id 11, not PPV). PPV=none. Attach status=attached. Flag status=entered-in-ai.</t>
+          <t>Finished bill (Invoice_Type 3). Header PO set=58948. Select Receipts 24283 2@146.5 on PO 58948. Invoice #=0040414821 (exact PDF). Amount=293.0 after-tax (never merchandise subtotal). Fees=none (Additional Charge Fees id 11, not PPV). PPV=none. Attach status=attached. Finish Select Receipts selected ids=[24283] fees=none ppv=none. Flag status=entered-in-ai.</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr"/>
       <c r="I11" s="2" t="inlineStr"/>
       <c r="J11" s="2" t="n">
-        <v>10135</v>
+        <v>10137</v>
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
@@ -1226,7 +1210,7 @@
       </c>
       <c r="L11" s="2" t="inlineStr">
         <is>
-          <t>$SUR485005 1 0 FUEL SURCHARGE EA 17.50 17.50 N 17.5</t>
+          <t>none</t>
         </is>
       </c>
       <c r="M11" s="2" t="inlineStr">
@@ -1259,32 +1243,44 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>0040438494</t>
+          <t>0040430010</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr"/>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>59081</t>
+        </is>
+      </c>
       <c r="E12" s="2" t="n">
-        <v>331.5</v>
-      </c>
-      <c r="F12" s="3" t="inlineStr">
-        <is>
-          <t>Success</t>
+        <v>14</v>
+      </c>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>HOLD</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Finished bill (Invoice_Type 4). Header PO set=none. Misc Type 4 Lines-K Shop Supplies - G&amp;S (no PO). Invoice #=0040438494 (exact PDF). Amount=331.5 after-tax (never merchandise subtotal). Fees=$SUR485005 1 0 FUEL SURCHARGE EA 17.50 17.50 N 17.5 (Additional Charge Fees id 11, not PPV). PPV=none. Attach status=attached. Flag status=entered-in-ai.</t>
-        </is>
-      </c>
-      <c r="H12" s="2" t="inlineStr"/>
-      <c r="I12" s="2" t="inlineStr"/>
+          <t>category=missing_receipt; owner=Ruben Perez. HOLD (receipt): no open receipt leftover on PO 59081 for Gas and Supply invoice #0040430010. PDF merch=MLW49-56-7240 1.0@14.0; selected=none. Do not first-open guess. Do not invent Success. @Ruben Perez: receiving must receive the PO so AP can Select Receipts. Parent email will be Entered with issues. Outlook Entered with issues. Flag status=entered-with-issues.</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>missing_receipt</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>Ruben Perez</t>
+        </is>
+      </c>
       <c r="J12" s="2" t="n">
-        <v>10136</v>
+        <v>10165</v>
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
@@ -1293,7 +1289,7 @@
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>$SUR485005 1 0 FUEL SURCHARGE EA 17.50 17.50 N 17.5</t>
+          <t>none</t>
         </is>
       </c>
       <c r="M12" s="2" t="inlineStr">
@@ -1326,12 +1322,12 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>0040438057</t>
+          <t>0040424839</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
@@ -1340,7 +1336,7 @@
         </is>
       </c>
       <c r="E13" s="2" t="n">
-        <v>36.12</v>
+        <v>224.94</v>
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
@@ -1349,20 +1345,22 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>category=missing_po; owner=Shawn McKibben. HOLD (po): PO 59081 is on the invoice but not findable on live by vendor + part/WO. Will not enter as Misc Type 4 (Willbanks 209663/209664; RMP 1470159). multi-invoice-pdf page 1–2 of 7</t>
+          <t>category=missing_receipt; owner=Ruben Perez. HOLD (receipt): no open receipt leftover on PO 59081 for Gas and Supply invoice #0040424839. PDF merch=GHS4000A 3.0@11.3; STY57-533A 4.0@47.76; selected=none. Do not first-open guess. Do not invent Success. @Ruben Perez: receiving must receive the PO so AP can Select Receipts. Parent email will be Entered with issues. Outlook Entered with issues. Flag status=entered-with-issues.</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>missing_po</t>
+          <t>missing_receipt</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>Shawn McKibben</t>
-        </is>
-      </c>
-      <c r="J13" s="2" t="inlineStr"/>
+          <t>Ruben Perez</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="n">
+        <v>10166</v>
+      </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
           <t>API Agent - 9/17/26 Gas &amp; Supply (720)</t>
@@ -1380,7 +1378,7 @@
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>pdf-on-vm</t>
+          <t>attached</t>
         </is>
       </c>
       <c r="O13" s="2" t="inlineStr">
@@ -1403,7 +1401,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>0040438056</t>
+          <t>0040438057</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -1417,7 +1415,7 @@
         </is>
       </c>
       <c r="E14" s="2" t="n">
-        <v>207.53</v>
+        <v>36.12</v>
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
@@ -1426,20 +1424,22 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>category=missing_po; owner=Shawn McKibben. HOLD (po): PO 59081 is on the invoice but not findable on live by vendor + part/WO. Will not enter as Misc Type 4 (Willbanks 209663/209664; RMP 1470159). multi-invoice-pdf page 7–8 of 7</t>
+          <t>category=missing_receipt; owner=Ruben Perez. HOLD (receipt): no open receipt leftover on PO 59081 for Gas and Supply invoice #0040438057. PDF merch=PFXPXTW1425R 1.0@36.12; selected=none. Do not first-open guess. Do not invent Success. @Ruben Perez: receiving must receive the PO so AP can Select Receipts. Parent email will be Entered with issues. Outlook Entered with issues. Flag status=entered-with-issues.</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>missing_po</t>
+          <t>missing_receipt</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>Shawn McKibben</t>
-        </is>
-      </c>
-      <c r="J14" s="2" t="inlineStr"/>
+          <t>Ruben Perez</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="n">
+        <v>10167</v>
+      </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
           <t>API Agent - 9/17/26 Gas &amp; Supply (720)</t>
@@ -1457,7 +1457,7 @@
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>pdf-on-vm</t>
+          <t>attached</t>
         </is>
       </c>
       <c r="O14" s="2" t="inlineStr">
@@ -1480,7 +1480,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>0040438055</t>
+          <t>0040438056</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -1494,7 +1494,7 @@
         </is>
       </c>
       <c r="E15" s="2" t="n">
-        <v>27.82</v>
+        <v>207.53</v>
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
@@ -1503,20 +1503,22 @@
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>category=missing_po; owner=Shawn McKibben. HOLD (po): PO 59081 is on the invoice but not findable on live by vendor + part/WO. Will not enter as Misc Type 4 (Willbanks 209663/209664; RMP 1470159). multi-invoice-pdf page 8–8 of 7</t>
+          <t>category=missing_receipt; owner=Ruben Perez. HOLD (receipt): no open receipt leftover on PO 59081 for Gas and Supply invoice #0040438056. PDF merch=MIL269767 1.0@108.82; MIL269771 1.0@98.71; selected=none. Do not first-open guess. Do not invent Success. @Ruben Perez: receiving must receive the PO so AP can Select Receipts. Parent email will be Entered with issues. Outlook Entered with issues. Flag status=entered-with-issues.</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>missing_po</t>
+          <t>missing_receipt</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>Shawn McKibben</t>
-        </is>
-      </c>
-      <c r="J15" s="2" t="inlineStr"/>
+          <t>Ruben Perez</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="n">
+        <v>10168</v>
+      </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
           <t>API Agent - 9/17/26 Gas &amp; Supply (720)</t>
@@ -1534,7 +1536,7 @@
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>pdf-on-vm</t>
+          <t>attached</t>
         </is>
       </c>
       <c r="O15" s="2" t="inlineStr">
@@ -1557,7 +1559,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>0040438053</t>
+          <t>0040438055</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -1571,7 +1573,7 @@
         </is>
       </c>
       <c r="E16" s="2" t="n">
-        <v>182.5</v>
+        <v>27.82</v>
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
@@ -1580,20 +1582,22 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>category=missing_po; owner=Shawn McKibben. HOLD (po): PO 59081 is on the invoice but not findable on live by vendor + part/WO. Will not enter as Misc Type 4 (Willbanks 209663/209664; RMP 1470159). multi-invoice-pdf page 6–7 of 7</t>
+          <t>category=missing_receipt; owner=Ruben Perez. HOLD (receipt): no open receipt leftover on PO 59081 for Gas and Supply invoice #0040438055. PDF merch=PRTJ7324H 2.0@13.91; selected=none. Do not first-open guess. Do not invent Success. @Ruben Perez: receiving must receive the PO so AP can Select Receipts. Parent email will be Entered with issues. Outlook Entered with issues. Flag status=entered-with-issues.</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>missing_po</t>
+          <t>missing_receipt</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>Shawn McKibben</t>
-        </is>
-      </c>
-      <c r="J16" s="2" t="inlineStr"/>
+          <t>Ruben Perez</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="n">
+        <v>10169</v>
+      </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
           <t>API Agent - 9/17/26 Gas &amp; Supply (720)</t>
@@ -1611,7 +1615,7 @@
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
-          <t>pdf-on-vm</t>
+          <t>attached</t>
         </is>
       </c>
       <c r="O16" s="2" t="inlineStr">
@@ -1634,12 +1638,12 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>0040417672</t>
+          <t>0040438053</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
@@ -1648,7 +1652,7 @@
         </is>
       </c>
       <c r="E17" s="2" t="n">
-        <v>3856.77</v>
+        <v>182.5</v>
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
@@ -1657,20 +1661,22 @@
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>category=missing_po; owner=Shawn McKibben. HOLD (po): PO 59081 is on the invoice but not findable on live by vendor + part/WO. Will not enter as Misc Type 4 (Willbanks 209663/209664; RMP 1470159).</t>
+          <t>category=missing_receipt; owner=Ruben Perez. HOLD (receipt): no open receipt leftover on PO 59081 for Gas and Supply invoice #0040438053. PDF merch=ELCWW10204F-DP 1.0@182.5; selected=none. Do not first-open guess. Do not invent Success. @Ruben Perez: receiving must receive the PO so AP can Select Receipts. Parent email will be Entered with issues. Outlook Entered with issues. Flag status=entered-with-issues.</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>missing_po</t>
+          <t>missing_receipt</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>Shawn McKibben</t>
-        </is>
-      </c>
-      <c r="J17" s="2" t="inlineStr"/>
+          <t>Ruben Perez</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="n">
+        <v>10170</v>
+      </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
           <t>API Agent - 9/17/26 Gas &amp; Supply (720)</t>
@@ -1688,7 +1694,7 @@
       </c>
       <c r="N17" s="2" t="inlineStr">
         <is>
-          <t>pdf-on-vm</t>
+          <t>attached</t>
         </is>
       </c>
       <c r="O17" s="2" t="inlineStr">
@@ -1698,7 +1704,7 @@
       </c>
       <c r="P17" s="2" t="inlineStr">
         <is>
-          <t>ai-hold</t>
+          <t>entered-with-issues</t>
         </is>
       </c>
       <c r="Q17" s="2" t="inlineStr"/>
@@ -1711,21 +1717,21 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>0040414962</t>
+          <t>0040417672</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>59006</t>
+          <t>59081</t>
         </is>
       </c>
       <c r="E18" s="2" t="n">
-        <v>7840.8</v>
+        <v>3856.77</v>
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
@@ -1734,20 +1740,22 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>category=missing_po; owner=Shawn McKibben. HOLD (po): PO 59006 is on the invoice but not findable on live by vendor + part/WO. Will not enter as Misc Type 4 (Willbanks 209663/209664; RMP 1470159). multi-invoice-pdf page 2–2 of 2</t>
+          <t>category=missing_receipt; owner=Ruben Perez. HOLD (receipt): no open receipt leftover on PO 59081 for Gas and Supply invoice #0040417672. PDF merch=CGW42304 100.0@3.88; 3-M60440227472 200.0@5.25; WSP1801S0020 48.0@5.5; PFXPX23T37 60.0@9.63; PFXPX14H35 250.0@0.87; PFXPX14H45 250.0@0.97; TIL48M 12.0@15.96; PIP34-874/XL 48.0@4.68; MKL96007 4.0@6.44; MIL269765 1.0@184.04; MIL301253 1.0@180.18; PFXPXTW1425R 1.0@36.12; STY54-024 3.0@18.83; ANC30SS 50.0@1.24; VIC0323-0252 2.0@78.37; selected=none. Do not first-open guess. Do not invent Success. @Ruben Perez: receiving must receive the PO so AP can Select Receipts. Parent email will be Entered with issues. Outlook Entered with issues. Flag status=entered-with-issues.</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>missing_po</t>
+          <t>missing_receipt</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>Shawn McKibben</t>
-        </is>
-      </c>
-      <c r="J18" s="2" t="inlineStr"/>
+          <t>Ruben Perez</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="n">
+        <v>10171</v>
+      </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
           <t>API Agent - 9/17/26 Gas &amp; Supply (720)</t>
@@ -1765,7 +1773,7 @@
       </c>
       <c r="N18" s="2" t="inlineStr">
         <is>
-          <t>pdf-on-vm</t>
+          <t>attached</t>
         </is>
       </c>
       <c r="O18" s="2" t="inlineStr">
@@ -1788,7 +1796,7 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>0040414821</t>
+          <t>0040414962</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
@@ -1798,26 +1806,34 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>58948</t>
+          <t>59006</t>
         </is>
       </c>
       <c r="E19" s="2" t="n">
-        <v>293</v>
-      </c>
-      <c r="F19" s="3" t="inlineStr">
-        <is>
-          <t>Success</t>
+        <v>7840.8</v>
+      </c>
+      <c r="F19" s="4" t="inlineStr">
+        <is>
+          <t>HOLD</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>Finished bill (Invoice_Type 3). Header PO set=58948. Select Receipts 24283 2@146.5 on PO 58948. Invoice #=0040414821 (exact PDF). Amount=293.0 after-tax (never merchandise subtotal). Fees=none (Additional Charge Fees id 11, not PPV). PPV=none. Attach status=attached. Finish Select Receipts selected ids=[24283] fees=none ppv=none. Flag status=entered-in-ai.</t>
-        </is>
-      </c>
-      <c r="H19" s="2" t="inlineStr"/>
-      <c r="I19" s="2" t="inlineStr"/>
+          <t>category=missing_receipt; owner=Ruben Perez. HOLD (receipt): no open receipt leftover on PO 59006 for Gas and Supply invoice #0040414962. PDF merch=LINEDS30778 880.0@8.91; selected=none. Do not first-open guess. Do not invent Success. @Ruben Perez: receiving must receive the PO so AP can Select Receipts. Parent email will be Entered with issues. Outlook Entered with issues. Flag status=entered-with-issues.</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>missing_receipt</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>Ruben Perez</t>
+        </is>
+      </c>
       <c r="J19" s="2" t="n">
-        <v>10137</v>
+        <v>10172</v>
       </c>
       <c r="K19" s="2" t="inlineStr">
         <is>
@@ -1846,7 +1862,7 @@
       </c>
       <c r="P19" s="2" t="inlineStr">
         <is>
-          <t>entered-in-ai</t>
+          <t>entered-with-issues</t>
         </is>
       </c>
       <c r="Q19" s="2" t="inlineStr"/>
@@ -1885,7 +1901,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>missing_po</t>
+          <t>missing_receipt</t>
         </is>
       </c>
       <c r="B2" t="n">

</xml_diff>

<commit_message>
Record Gas 10165-10172 Success after Shawn 59081/59006 receive.
Live GET-prove: Type 3 on batch 720, Amount=Verification=PDF, receipts
selected. 0040417672 posted in-gate PPV -0.52. No Mail.Send.

Co-authored-by: beave89atm <beave89atm@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/runs/AP-run-2026-09-17-gas-supply.xlsx
+++ b/runs/AP-run-2026-09-17-gas-supply.xlsx
@@ -33,7 +33,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -50,11 +50,6 @@
         <fgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFEB9C"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -68,7 +63,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
@@ -77,9 +72,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -1259,26 +1251,18 @@
       <c r="E12" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="F12" s="4" t="inlineStr">
-        <is>
-          <t>HOLD</t>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>Success</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>category=missing_receipt; owner=Ruben Perez. HOLD (receipt): no open receipt leftover on PO 59081 for Gas and Supply invoice #0040430010. PDF merch=MLW49-56-7240 1.0@14.0; selected=none. Do not first-open guess. Do not invent Success. @Ruben Perez: receiving must receive the PO so AP can Select Receipts. Parent email will be Entered with issues. Outlook Entered with issues. Flag status=entered-with-issues.</t>
-        </is>
-      </c>
-      <c r="H12" s="2" t="inlineStr">
-        <is>
-          <t>missing_receipt</t>
-        </is>
-      </c>
-      <c r="I12" s="2" t="inlineStr">
-        <is>
-          <t>Ruben Perez</t>
-        </is>
-      </c>
+          <t>Finished bill (Invoice_Type 3). Header PO set=59081. Select Receipts 24333 1@14.0 on PO 59081. Invoice #=0040430010 (exact PDF). Amount=14.0 after-tax (never merchandise subtotal). Fees=none (Additional Charge Fees id 11, not PPV). PPV=none. Attach status=attached. Finish Select Receipts selected ids=[24333] fees=none ppv=none. Flag status=entered-in-ai.</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr"/>
+      <c r="I12" s="2" t="inlineStr"/>
       <c r="J12" s="2" t="n">
         <v>10165</v>
       </c>
@@ -1309,7 +1293,7 @@
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>entered-with-issues</t>
+          <t>entered-in-ai</t>
         </is>
       </c>
       <c r="Q12" s="2" t="inlineStr"/>
@@ -1338,26 +1322,18 @@
       <c r="E13" s="2" t="n">
         <v>224.94</v>
       </c>
-      <c r="F13" s="4" t="inlineStr">
-        <is>
-          <t>HOLD</t>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>Success</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>category=missing_receipt; owner=Ruben Perez. HOLD (receipt): no open receipt leftover on PO 59081 for Gas and Supply invoice #0040424839. PDF merch=GHS4000A 3.0@11.3; STY57-533A 4.0@47.76; selected=none. Do not first-open guess. Do not invent Success. @Ruben Perez: receiving must receive the PO so AP can Select Receipts. Parent email will be Entered with issues. Outlook Entered with issues. Flag status=entered-with-issues.</t>
-        </is>
-      </c>
-      <c r="H13" s="2" t="inlineStr">
-        <is>
-          <t>missing_receipt</t>
-        </is>
-      </c>
-      <c r="I13" s="2" t="inlineStr">
-        <is>
-          <t>Ruben Perez</t>
-        </is>
-      </c>
+          <t>Finished bill (Invoice_Type 3). Header PO set=59081. Select Receipts 24334 3@11.3; 24335 4@47.76 on PO 59081. Invoice #=0040424839 (exact PDF). Amount=224.94 after-tax (never merchandise subtotal). Fees=none (Additional Charge Fees id 11, not PPV). PPV=none. Attach status=attached. Finish Select Receipts selected ids=[24334, 24335] fees=none ppv=none. Flag status=entered-in-ai.</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr"/>
+      <c r="I13" s="2" t="inlineStr"/>
       <c r="J13" s="2" t="n">
         <v>10166</v>
       </c>
@@ -1388,7 +1364,7 @@
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>entered-with-issues</t>
+          <t>entered-in-ai</t>
         </is>
       </c>
       <c r="Q13" s="2" t="inlineStr"/>
@@ -1417,26 +1393,18 @@
       <c r="E14" s="2" t="n">
         <v>36.12</v>
       </c>
-      <c r="F14" s="4" t="inlineStr">
-        <is>
-          <t>HOLD</t>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>Success</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>category=missing_receipt; owner=Ruben Perez. HOLD (receipt): no open receipt leftover on PO 59081 for Gas and Supply invoice #0040438057. PDF merch=PFXPXTW1425R 1.0@36.12; selected=none. Do not first-open guess. Do not invent Success. @Ruben Perez: receiving must receive the PO so AP can Select Receipts. Parent email will be Entered with issues. Outlook Entered with issues. Flag status=entered-with-issues.</t>
-        </is>
-      </c>
-      <c r="H14" s="2" t="inlineStr">
-        <is>
-          <t>missing_receipt</t>
-        </is>
-      </c>
-      <c r="I14" s="2" t="inlineStr">
-        <is>
-          <t>Ruben Perez</t>
-        </is>
-      </c>
+          <t>Finished bill (Invoice_Type 3). Header PO set=59081. Select Receipts 24336 1@36.12 on PO 59081. Invoice #=0040438057 (exact PDF). Amount=36.12 after-tax (never merchandise subtotal). Fees=none (Additional Charge Fees id 11, not PPV). PPV=none. Attach status=attached. Finish Select Receipts selected ids=[24336] fees=none ppv=none. Flag status=entered-in-ai.</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr"/>
+      <c r="I14" s="2" t="inlineStr"/>
       <c r="J14" s="2" t="n">
         <v>10167</v>
       </c>
@@ -1467,7 +1435,7 @@
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>entered-with-issues</t>
+          <t>entered-in-ai</t>
         </is>
       </c>
       <c r="Q14" s="2" t="inlineStr"/>
@@ -1496,26 +1464,18 @@
       <c r="E15" s="2" t="n">
         <v>207.53</v>
       </c>
-      <c r="F15" s="4" t="inlineStr">
-        <is>
-          <t>HOLD</t>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>Success</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>category=missing_receipt; owner=Ruben Perez. HOLD (receipt): no open receipt leftover on PO 59081 for Gas and Supply invoice #0040438056. PDF merch=MIL269767 1.0@108.82; MIL269771 1.0@98.71; selected=none. Do not first-open guess. Do not invent Success. @Ruben Perez: receiving must receive the PO so AP can Select Receipts. Parent email will be Entered with issues. Outlook Entered with issues. Flag status=entered-with-issues.</t>
-        </is>
-      </c>
-      <c r="H15" s="2" t="inlineStr">
-        <is>
-          <t>missing_receipt</t>
-        </is>
-      </c>
-      <c r="I15" s="2" t="inlineStr">
-        <is>
-          <t>Ruben Perez</t>
-        </is>
-      </c>
+          <t>Finished bill (Invoice_Type 3). Header PO set=59081. Select Receipts 24337 1@108.82; 24338 1@98.71 on PO 59081. Invoice #=0040438056 (exact PDF). Amount=207.53 after-tax (never merchandise subtotal). Fees=none (Additional Charge Fees id 11, not PPV). PPV=none. Attach status=attached. Finish Select Receipts selected ids=[24337, 24338] fees=none ppv=none. Flag status=entered-in-ai.</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr"/>
+      <c r="I15" s="2" t="inlineStr"/>
       <c r="J15" s="2" t="n">
         <v>10168</v>
       </c>
@@ -1546,7 +1506,7 @@
       </c>
       <c r="P15" s="2" t="inlineStr">
         <is>
-          <t>entered-with-issues</t>
+          <t>entered-in-ai</t>
         </is>
       </c>
       <c r="Q15" s="2" t="inlineStr"/>
@@ -1575,26 +1535,18 @@
       <c r="E16" s="2" t="n">
         <v>27.82</v>
       </c>
-      <c r="F16" s="4" t="inlineStr">
-        <is>
-          <t>HOLD</t>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>Success</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>category=missing_receipt; owner=Ruben Perez. HOLD (receipt): no open receipt leftover on PO 59081 for Gas and Supply invoice #0040438055. PDF merch=PRTJ7324H 2.0@13.91; selected=none. Do not first-open guess. Do not invent Success. @Ruben Perez: receiving must receive the PO so AP can Select Receipts. Parent email will be Entered with issues. Outlook Entered with issues. Flag status=entered-with-issues.</t>
-        </is>
-      </c>
-      <c r="H16" s="2" t="inlineStr">
-        <is>
-          <t>missing_receipt</t>
-        </is>
-      </c>
-      <c r="I16" s="2" t="inlineStr">
-        <is>
-          <t>Ruben Perez</t>
-        </is>
-      </c>
+          <t>Finished bill (Invoice_Type 3). Header PO set=59081. Select Receipts 24339 2@13.91 on PO 59081. Invoice #=0040438055 (exact PDF). Amount=27.82 after-tax (never merchandise subtotal). Fees=none (Additional Charge Fees id 11, not PPV). PPV=none. Attach status=attached. Finish Select Receipts selected ids=[24339] fees=none ppv=none. Flag status=entered-in-ai.</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr"/>
+      <c r="I16" s="2" t="inlineStr"/>
       <c r="J16" s="2" t="n">
         <v>10169</v>
       </c>
@@ -1625,7 +1577,7 @@
       </c>
       <c r="P16" s="2" t="inlineStr">
         <is>
-          <t>entered-with-issues</t>
+          <t>entered-in-ai</t>
         </is>
       </c>
       <c r="Q16" s="2" t="inlineStr"/>
@@ -1654,26 +1606,18 @@
       <c r="E17" s="2" t="n">
         <v>182.5</v>
       </c>
-      <c r="F17" s="4" t="inlineStr">
-        <is>
-          <t>HOLD</t>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>Success</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>category=missing_receipt; owner=Ruben Perez. HOLD (receipt): no open receipt leftover on PO 59081 for Gas and Supply invoice #0040438053. PDF merch=ELCWW10204F-DP 1.0@182.5; selected=none. Do not first-open guess. Do not invent Success. @Ruben Perez: receiving must receive the PO so AP can Select Receipts. Parent email will be Entered with issues. Outlook Entered with issues. Flag status=entered-with-issues.</t>
-        </is>
-      </c>
-      <c r="H17" s="2" t="inlineStr">
-        <is>
-          <t>missing_receipt</t>
-        </is>
-      </c>
-      <c r="I17" s="2" t="inlineStr">
-        <is>
-          <t>Ruben Perez</t>
-        </is>
-      </c>
+          <t>Finished bill (Invoice_Type 3). Header PO set=59081. Select Receipts 24340 1@182.5 on PO 59081. Invoice #=0040438053 (exact PDF). Amount=182.5 after-tax (never merchandise subtotal). Fees=none (Additional Charge Fees id 11, not PPV). PPV=none. Attach status=attached. Finish Select Receipts selected ids=[24340] fees=none ppv=none. Flag status=entered-in-ai.</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr"/>
+      <c r="I17" s="2" t="inlineStr"/>
       <c r="J17" s="2" t="n">
         <v>10170</v>
       </c>
@@ -1704,7 +1648,7 @@
       </c>
       <c r="P17" s="2" t="inlineStr">
         <is>
-          <t>entered-with-issues</t>
+          <t>entered-in-ai</t>
         </is>
       </c>
       <c r="Q17" s="2" t="inlineStr"/>
@@ -1733,26 +1677,18 @@
       <c r="E18" s="2" t="n">
         <v>3856.77</v>
       </c>
-      <c r="F18" s="4" t="inlineStr">
-        <is>
-          <t>HOLD</t>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>Success</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>category=missing_receipt; owner=Ruben Perez. HOLD (receipt): no open receipt leftover on PO 59081 for Gas and Supply invoice #0040417672. PDF merch=CGW42304 100.0@3.88; 3-M60440227472 200.0@5.25; WSP1801S0020 48.0@5.5; PFXPX23T37 60.0@9.63; PFXPX14H35 250.0@0.87; PFXPX14H45 250.0@0.97; TIL48M 12.0@15.96; PIP34-874/XL 48.0@4.68; MKL96007 4.0@6.44; MIL269765 1.0@184.04; MIL301253 1.0@180.18; PFXPXTW1425R 1.0@36.12; STY54-024 3.0@18.83; ANC30SS 50.0@1.24; VIC0323-0252 2.0@78.37; selected=none. Do not first-open guess. Do not invent Success. @Ruben Perez: receiving must receive the PO so AP can Select Receipts. Parent email will be Entered with issues. Outlook Entered with issues. Flag status=entered-with-issues.</t>
-        </is>
-      </c>
-      <c r="H18" s="2" t="inlineStr">
-        <is>
-          <t>missing_receipt</t>
-        </is>
-      </c>
-      <c r="I18" s="2" t="inlineStr">
-        <is>
-          <t>Ruben Perez</t>
-        </is>
-      </c>
+          <t>Finished bill (Invoice_Type 3). Header PO set=59081. Select Receipts 24341 100@3.88; 24350 1@184.04; 24351 1@180.18; 24352 1@36.12; 24353 3@18.83; 24354 50@1.24; 24355 2@78.37; 24342 200@5.25; 24343 48@5.5; 24344 60@9.63; 24345 250@0.87; 24346 250@0.97; 24347 12@15.96; 24348 48@4.68; 24349 4@6.44 on PO 59081. Invoice #=0040417672 (exact PDF). Amount=3856.77 after-tax (never merchandise subtotal). Fees=none (Additional Charge Fees id 11, not PPV). PPV=-0.52. Attach status=attached. Finish Select Receipts selected ids=[24341, 24342, 24343, 24344, 24345, 24346, 24347, 24348, 24349, 24350, 24351, 24352, 24353, 24354, 24355] fees=none ppv=posted. Flag status=entered-in-ai.</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr"/>
+      <c r="I18" s="2" t="inlineStr"/>
       <c r="J18" s="2" t="n">
         <v>10171</v>
       </c>
@@ -1768,7 +1704,7 @@
       </c>
       <c r="M18" s="2" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>-0.52</t>
         </is>
       </c>
       <c r="N18" s="2" t="inlineStr">
@@ -1783,7 +1719,7 @@
       </c>
       <c r="P18" s="2" t="inlineStr">
         <is>
-          <t>entered-with-issues</t>
+          <t>entered-in-ai</t>
         </is>
       </c>
       <c r="Q18" s="2" t="inlineStr"/>
@@ -1812,26 +1748,18 @@
       <c r="E19" s="2" t="n">
         <v>7840.8</v>
       </c>
-      <c r="F19" s="4" t="inlineStr">
-        <is>
-          <t>HOLD</t>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>Success</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>category=missing_receipt; owner=Ruben Perez. HOLD (receipt): no open receipt leftover on PO 59006 for Gas and Supply invoice #0040414962. PDF merch=LINEDS30778 880.0@8.91; selected=none. Do not first-open guess. Do not invent Success. @Ruben Perez: receiving must receive the PO so AP can Select Receipts. Parent email will be Entered with issues. Outlook Entered with issues. Flag status=entered-with-issues.</t>
-        </is>
-      </c>
-      <c r="H19" s="2" t="inlineStr">
-        <is>
-          <t>missing_receipt</t>
-        </is>
-      </c>
-      <c r="I19" s="2" t="inlineStr">
-        <is>
-          <t>Ruben Perez</t>
-        </is>
-      </c>
+          <t>Finished bill (Invoice_Type 3). Header PO set=59006. Select Receipts 24332 880@8.91 on PO 59006. Invoice #=0040414962 (exact PDF). Amount=7840.8 after-tax (never merchandise subtotal). Fees=none (Additional Charge Fees id 11, not PPV). PPV=none. Attach status=attached. Finish Select Receipts selected ids=[24332] fees=none ppv=none. Flag status=entered-in-ai.</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr"/>
+      <c r="I19" s="2" t="inlineStr"/>
       <c r="J19" s="2" t="n">
         <v>10172</v>
       </c>
@@ -1862,7 +1790,7 @@
       </c>
       <c r="P19" s="2" t="inlineStr">
         <is>
-          <t>entered-with-issues</t>
+          <t>entered-in-ai</t>
         </is>
       </c>
       <c r="Q19" s="2" t="inlineStr"/>
@@ -1879,7 +1807,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:B1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1887,25 +1815,15 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="inlineStr">
+      <c r="A1" s="4" t="inlineStr">
         <is>
           <t>Exception category</t>
         </is>
       </c>
-      <c r="B1" s="5" t="inlineStr">
+      <c r="B1" s="4" t="inlineStr">
         <is>
           <t>Count</t>
         </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>missing_receipt</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Record Gas 0040438052 entered as 10173 HOLD missing_receipt.
9/17 multi-invoice PDF (received 2026-09-18T04:46Z) listed seven invoices.
0040438052 was the leftover after plus-10 cap; now on batch 720 Type 3
PO 59081 with pages 5–6 only. LINEDS01162 500@10.36 has no open leftover.
Gas owner blank — no @tag. Parent stays Entered with issues (0040437952 still out).

Co-authored-by: beave89atm <beave89atm@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/runs/AP-run-2026-09-17-gas-supply.xlsx
+++ b/runs/AP-run-2026-09-17-gas-supply.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Exception counts" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'AP run'!$A$1:$Q$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'AP run'!$A$1:$Q$20</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -33,7 +33,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -50,6 +50,11 @@
         <fgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFEB9C"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -63,7 +68,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
@@ -72,6 +77,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -440,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q19"/>
+  <dimension ref="A1:Q20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1795,8 +1803,87 @@
       </c>
       <c r="Q19" s="2" t="inlineStr"/>
     </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>Gas and Supply North Texas, LLC</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>0040438052</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>59081</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="n">
+        <v>5178.55</v>
+      </c>
+      <c r="F20" s="4" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>category=missing_receipt; owner=none (Gas receiving owner blank). HOLD (receipt): no open receipt leftover on PO 59081 for Gas and Supply invoice #0040438052. PDF merch=LINEDS01162 500.0@10.36; selected=none. Do not first-open guess. Do not invent Success. no receiving @tag (Gas owner blank): receiving must receive the PO so AP can Select Receipts. Parent email will be Entered with issues. Outlook Entered with issues. Flag status=entered-with-issues.</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>missing_receipt</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>none (Gas receiving owner blank)</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="n">
+        <v>10173</v>
+      </c>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t>API Agent - 9/17/26 Gas &amp; Supply (720)</t>
+        </is>
+      </c>
+      <c r="L20" s="2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="M20" s="2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="N20" s="2" t="inlineStr">
+        <is>
+          <t>attached</t>
+        </is>
+      </c>
+      <c r="O20" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P20" s="2" t="inlineStr">
+        <is>
+          <t>entered-with-issues</t>
+        </is>
+      </c>
+      <c r="Q20" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:Q19"/>
+  <autoFilter ref="A1:Q20"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1807,7 +1894,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1"/>
+  <dimension ref="A1:B2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1815,15 +1902,25 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" s="5" t="inlineStr">
         <is>
           <t>Exception category</t>
         </is>
       </c>
-      <c r="B1" s="4" t="inlineStr">
+      <c r="B1" s="5" t="inlineStr">
         <is>
           <t>Count</t>
         </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>missing_receipt</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Record Gas 0040437952 as 10181 HOLD missing_receipt on 720.
Entered Type 3 PO 59006 with pages 4–5. First-open wrongly selected
24332 (10172 LINEDS30778); deselected and returned from Transfer AP.
PDF merch DEWDW1969 3@80.49 has no leftover. No receiving @tag.
Parent Outlook stays Entered with issues (0040438052 still HOLD).

Co-authored-by: beave89atm <beave89atm@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/runs/AP-run-2026-09-17-gas-supply.xlsx
+++ b/runs/AP-run-2026-09-17-gas-supply.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Exception counts" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'AP run'!$A$1:$Q$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'AP run'!$A$1:$Q$21</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q20"/>
+  <dimension ref="A1:Q21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1882,8 +1882,87 @@
       </c>
       <c r="Q20" s="2" t="inlineStr"/>
     </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Gas and Supply North Texas, LLC</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>0040437952</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>59006</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="n">
+        <v>241.46</v>
+      </c>
+      <c r="F21" s="4" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>category=missing_receipt; owner=none (Gas receiving owner blank). HOLD (receipt): PDF merch=DEWDW1969 3.0@80.49; leftover 24332 880@8.91 LINEDS30778 is 10172 / 0040414962 — first-open guess deselected. No matching leftover on PO 59006. Stay on batch 720. Do not @tag. Do not invent Success. Outlook Entered with issues (NOTE-51: sibling 0040438052 / 10173 still HOLD).</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>missing_receipt</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>none (Gas receiving owner blank)</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="n">
+        <v>10181</v>
+      </c>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>API Agent - 9/17/26 Gas &amp; Supply (720)</t>
+        </is>
+      </c>
+      <c r="L21" s="2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="M21" s="2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="N21" s="2" t="inlineStr">
+        <is>
+          <t>attached</t>
+        </is>
+      </c>
+      <c r="O21" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P21" s="2" t="inlineStr">
+        <is>
+          <t>entered-with-issues</t>
+        </is>
+      </c>
+      <c r="Q21" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:Q20"/>
+  <autoFilter ref="A1:Q21"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1920,7 +1999,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Record Shawn Comments_1 on Gas 10173/10181; keep both on 720.
10173 item 940 already persisted. 10181 restored 375→720 then item 941.
Sheet Exception owner set to Shawn McKibben. No Mail.Send.

Co-authored-by: beave89atm <beave89atm@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/runs/AP-run-2026-09-17-gas-supply.xlsx
+++ b/runs/AP-run-2026-09-17-gas-supply.xlsx
@@ -1834,7 +1834,7 @@
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>category=missing_receipt; owner=none (Gas receiving owner blank). HOLD (receipt): no open receipt leftover on PO 59081 for Gas and Supply invoice #0040438052. PDF merch=LINEDS01162 500.0@10.36; selected=none. Do not first-open guess. Do not invent Success. no receiving @tag (Gas owner blank): receiving must receive the PO so AP can Select Receipts. Parent email will be Entered with issues. Outlook Entered with issues. Flag status=entered-with-issues.</t>
+          <t>category=missing_receipt; owner=Shawn McKibben. Kyle 2026-09-22 override: ping Shawn on Gas missing_receipt (owner was blank). Comments_1 status=already-on-tab item_ids=[940] mention-id=104. Stay on API Agent - 9/17/26 Gas &amp; Supply (720). Do not Transfer AP. Do not invent Success. No Mail.Send. category=missing_receipt; owner=none (Gas receiving owner blank). HOLD (receipt): no open receipt leftover on PO 59081 for Gas and Supply invoice #0040438052. PDF merch=LINEDS01162 500.0@10.36; selected=none. Do not first-open guess. Do not invent Success. no receiving @tag (Gas owner blank): receiving must receive the PO so AP can Select Receipts. Parent email will be Entered with issues. Outlook Entered with issues. Flag status=entered-with-issues.</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
@@ -1844,7 +1844,7 @@
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>none (Gas receiving owner blank)</t>
+          <t>Shawn McKibben</t>
         </is>
       </c>
       <c r="J20" s="2" t="n">
@@ -1913,7 +1913,7 @@
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>category=missing_receipt; owner=none (Gas receiving owner blank). HOLD (receipt): PDF merch=DEWDW1969 3.0@80.49; leftover 24332 880@8.91 LINEDS30778 is 10172 / 0040414962 — first-open guess deselected. No matching leftover on PO 59006. Stay on batch 720. Do not @tag. Do not invent Success. Outlook Entered with issues (NOTE-51: sibling 0040438052 / 10173 still HOLD).</t>
+          <t>category=missing_receipt; owner=Shawn McKibben. Kyle 2026-09-22 override: ping Shawn on Gas missing_receipt (owner was blank). Comments_1 status=added item_ids=[941] mention-id=104. Stay on API Agent - 9/17/26 Gas &amp; Supply (720). Do not Transfer AP. Do not invent Success. No Mail.Send. category=missing_receipt; owner=none (Gas receiving owner blank). HOLD (receipt): PDF merch=DEWDW1969 3.0@80.49; leftover 24332 880@8.91 LINEDS30778 is 10172 / 0040414962 — first-open guess deselected. No matching leftover on PO 59006. Stay on batch 720. Do not @tag. Do not invent Success. Outlook Entered with issues (NOTE-51: sibling 0040438052 / 10173 still HOLD).</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
@@ -1923,7 +1923,7 @@
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>none (Gas receiving owner blank)</t>
+          <t>Shawn McKibben</t>
         </is>
       </c>
       <c r="J21" s="2" t="n">

</xml_diff>

<commit_message>
Record live NOTE-53 moves: 6 missing_receipt HOLDs to Transfer AP.
O'Neal 10160/10163/10175/10178 722→375. Gas 10173/10181 720→375.
Comments_1 kept (Anthony plain / Shawn 104). Sheets updated. No Mail.Send.

Co-authored-by: beave89atm <beave89atm@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/runs/AP-run-2026-09-17-gas-supply.xlsx
+++ b/runs/AP-run-2026-09-17-gas-supply.xlsx
@@ -1834,7 +1834,7 @@
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>category=missing_receipt; owner=Shawn McKibben. Kyle 2026-09-22 override: ping Shawn on Gas missing_receipt (owner was blank). Comments_1 status=already-on-tab item_ids=[940] mention-id=104. Stay on API Agent - 9/17/26 Gas &amp; Supply (720). Do not Transfer AP. Do not invent Success. No Mail.Send. category=missing_receipt; owner=none (Gas receiving owner blank). HOLD (receipt): no open receipt leftover on PO 59081 for Gas and Supply invoice #0040438052. PDF merch=LINEDS01162 500.0@10.36; selected=none. Do not first-open guess. Do not invent Success. no receiving @tag (Gas owner blank): receiving must receive the PO so AP can Select Receipts. Parent email will be Entered with issues. Outlook Entered with issues. Flag status=entered-with-issues.</t>
+          <t>category=missing_receipt; owner=Shawn McKibben. Kyle 2026-09-22 override: ping Shawn on Gas missing_receipt (owner was blank). Comments_1 status=already-on-tab item_ids=[940] mention-id=104. Stay on API Agent - 9/17/26 Gas &amp; Supply (720). Do not Transfer AP. Do not invent Success. No Mail.Send. category=missing_receipt; owner=none (Gas receiving owner blank). HOLD (receipt): no open receipt leftover on PO 59081 for Gas and Supply invoice #0040438052. PDF merch=LINEDS01162 500.0@10.36; selected=none. Do not first-open guess. Do not invent Success. no receiving @tag (Gas owner blank): receiving must receive the PO so AP can Select Receipts. Parent email will be Entered with issues. Outlook Entered with issues. Flag status=entered-with-issues. Kyle 2026-09-22 NOTE-53 missing_receipt → Transfer AP 720→375 status=moved.</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
@@ -1852,7 +1852,7 @@
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>API Agent - 9/17/26 Gas &amp; Supply (720)</t>
+          <t>Transfer AP (375)</t>
         </is>
       </c>
       <c r="L20" s="2" t="inlineStr">
@@ -1880,7 +1880,11 @@
           <t>entered-with-issues</t>
         </is>
       </c>
-      <c r="Q20" s="2" t="inlineStr"/>
+      <c r="Q20" s="2" t="inlineStr">
+        <is>
+          <t>Kyle 2026-09-22 NOTE-53 missing_receipt → Transfer AP 720→375 status=moved.</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1913,7 +1917,7 @@
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>category=missing_receipt; owner=Shawn McKibben. Kyle 2026-09-22 override: ping Shawn on Gas missing_receipt (owner was blank). Comments_1 status=added item_ids=[941] mention-id=104. Stay on API Agent - 9/17/26 Gas &amp; Supply (720). Do not Transfer AP. Do not invent Success. No Mail.Send. category=missing_receipt; owner=none (Gas receiving owner blank). HOLD (receipt): PDF merch=DEWDW1969 3.0@80.49; leftover 24332 880@8.91 LINEDS30778 is 10172 / 0040414962 — first-open guess deselected. No matching leftover on PO 59006. Stay on batch 720. Do not @tag. Do not invent Success. Outlook Entered with issues (NOTE-51: sibling 0040438052 / 10173 still HOLD).</t>
+          <t>category=missing_receipt; owner=Shawn McKibben. Kyle 2026-09-22 override: ping Shawn on Gas missing_receipt (owner was blank). Comments_1 status=added item_ids=[941] mention-id=104. Stay on API Agent - 9/17/26 Gas &amp; Supply (720). Do not Transfer AP. Do not invent Success. No Mail.Send. category=missing_receipt; owner=none (Gas receiving owner blank). HOLD (receipt): PDF merch=DEWDW1969 3.0@80.49; leftover 24332 880@8.91 LINEDS30778 is 10172 / 0040414962 — first-open guess deselected. No matching leftover on PO 59006. Stay on batch 720. Do not @tag. Do not invent Success. Outlook Entered with issues (NOTE-51: sibling 0040438052 / 10173 still HOLD). Kyle 2026-09-22 NOTE-53 missing_receipt → Transfer AP 720→375 status=moved.</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
@@ -1931,7 +1935,7 @@
       </c>
       <c r="K21" s="2" t="inlineStr">
         <is>
-          <t>API Agent - 9/17/26 Gas &amp; Supply (720)</t>
+          <t>Transfer AP (375)</t>
         </is>
       </c>
       <c r="L21" s="2" t="inlineStr">
@@ -1959,7 +1963,11 @@
           <t>entered-with-issues</t>
         </is>
       </c>
-      <c r="Q21" s="2" t="inlineStr"/>
+      <c r="Q21" s="2" t="inlineStr">
+        <is>
+          <t>Kyle 2026-09-22 NOTE-53 missing_receipt → Transfer AP 720→375 status=moved.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:Q21"/>

</xml_diff>

<commit_message>
Refresh O'Neal and Gas sheets after Fort Worth and Transfer AP.
Live GET batches: 10160/10163/10175/10178 + Gas 10173/10181 on TRANSFER AP 375.
Notes include NOTE-52 folder move and NOTE-53 batch move. 10162 stays price_variance/Shawn.

Co-authored-by: beave89atm <beave89atm@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/runs/AP-run-2026-09-17-gas-supply.xlsx
+++ b/runs/AP-run-2026-09-17-gas-supply.xlsx
@@ -8,7 +8,6 @@
   </bookViews>
   <sheets>
     <sheet name="AP run" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Exception counts" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'AP run'!$A$1:$Q$21</definedName>
@@ -68,7 +67,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
@@ -82,7 +81,6 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -467,10 +465,10 @@
     <col width="16" customWidth="1" min="14" max="14"/>
     <col width="18" customWidth="1" min="15" max="15"/>
     <col width="18" customWidth="1" min="16" max="16"/>
-    <col width="18" customWidth="1" min="17" max="17"/>
+    <col width="40" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22" customHeight="1">
+    <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Vendor</t>
@@ -1852,7 +1850,7 @@
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>Transfer AP (375)</t>
+          <t>TRANSFER AP (375)</t>
         </is>
       </c>
       <c r="L20" s="2" t="inlineStr">
@@ -1935,7 +1933,7 @@
       </c>
       <c r="K21" s="2" t="inlineStr">
         <is>
-          <t>Transfer AP (375)</t>
+          <t>TRANSFER AP (375)</t>
         </is>
       </c>
       <c r="L21" s="2" t="inlineStr">
@@ -1965,7 +1963,7 @@
       </c>
       <c r="Q21" s="2" t="inlineStr">
         <is>
-          <t>Kyle 2026-09-22 NOTE-53 missing_receipt → Transfer AP 720→375 status=moved.</t>
+          <t>Deselected 24332; returned from Transfer AP 375 to 720. Kyle 2026-09-22 NOTE-53 missing_receipt → Transfer AP 720→375 status=moved.</t>
         </is>
       </c>
     </row>
@@ -1973,44 +1971,4 @@
   <autoFilter ref="A1:Q21"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="5" t="inlineStr">
-        <is>
-          <t>Exception category</t>
-        </is>
-      </c>
-      <c r="B1" s="5" t="inlineStr">
-        <is>
-          <t>Count</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>missing_receipt</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>2</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>